<commit_message>
Revisão final: gap lido pelo nº de ECs (meses_operando contradiz data_inicio), rede 6,3 endereçáveis por EC, carga dos ECs da BA, KPI do tier Alta e textos corrigidos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/omie-case-contadores/output/Desafio2_Propensao.xlsx
+++ b/omie-case-contadores/output/Desafio2_Propensao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f75accf49a20a1b0/Documentos/Omie_Antigravity/omie-case-contadores/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_E86CD115D5B0E636EC0D9A4DCCF4E65D0BE23D50" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_286C251174ACDE36EC0D9A4DCCF4E65D0BE23D22" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -596,7 +596,7 @@
     <t>• Teste de estresse: com fator de realização = 0 (como o pipeline real sugere hoje), o uplift é zero — por isso o piloto.</t>
   </si>
   <si>
-    <t>• O nMRR da execução é 10 a 27x menor que o oficial das franquias; por isso o uplift % é o número principal (anexo SQL, A6/A7).</t>
+    <t>• O nMRR da execução é 10 a 27x menor que o oficial das franquias; por isso o uplift % é o número principal (franquias.realizado_nmrr_mes contra execucao_comercial.nmrr_gerado).</t>
   </si>
   <si>
     <t>id_contador</t>
@@ -4178,7 +4178,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FB62-41CC-A748-E035C4E5F1ED}"/>
+              <c16:uniqueId val="{00000000-FBEA-4850-956A-BAA48DD6143B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>